<commit_message>
Refresh the document ingestion control layer
A renamed snapshot of the control layer as of 2026-09-17, replacing the previous
snapshot. The client, every counterparty and every place are renamed, and no
production run, client record or personal data is included.
</commit_message>
<xml_diff>
--- a/examples/business_document_schema_samples.xlsx
+++ b/examples/business_document_schema_samples.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R0116e9182d064835"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extracted Sample" sheetId="2" r:id="Refeb95c5be774a01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived Controls" sheetId="3" r:id="R55c13b6591774d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM Adjudication" sheetId="4" r:id="R8fb0123e6c224e2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema Index" sheetId="5" r:id="Rc83e7fac19964052"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM Export" sheetId="6" r:id="Rf42e47245a504ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM Writes" sheetId="7" r:id="R498eb510a774488c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API and MCP" sheetId="8" r:id="R3f93467e36c34bb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connector Access" sheetId="9" r:id="Rbacd696a28fa411d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standard Reports" sheetId="10" r:id="R333c12b800154f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query Examples" sheetId="11" r:id="Rcc512e24d86a4a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visual Intake" sheetId="12" r:id="R29854b8beeb84e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R5f64ee5abc684472"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extracted Sample" sheetId="2" r:id="Rd70a4b16db6541a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derived Controls" sheetId="3" r:id="R8f74413a07ab47b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM Adjudication" sheetId="4" r:id="R479dc7c8591b4256"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema Index" sheetId="5" r:id="R884d4b3251f44a76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM Export" sheetId="6" r:id="Re125f6ec80d44524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM Writes" sheetId="7" r:id="Re879868154b349ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API and MCP" sheetId="8" r:id="R954e2b8fb35a4c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connector Access" sheetId="9" r:id="Ra4652340694d4dda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standard Reports" sheetId="10" r:id="R27851714b15548eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query Examples" sheetId="11" r:id="R5d06891028844764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visual Intake" sheetId="12" r:id="R7290d3a9fe164719"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -350,7 +350,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="ApiMcpCapabilitiesTable" displayName="ApiMcpCapabilitiesTable" ref="A4:E18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="ApiMcpCapabilitiesTable" displayName="ApiMcpCapabilitiesTable" ref="A4:E29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Function"/>
     <x:tableColumn id="2" name="HTTPS API"/>
@@ -390,7 +390,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="CrmQueryExamplesTable" displayName="CrmQueryExamplesTable" ref="A4:D12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="CrmQueryExamplesTable" displayName="CrmQueryExamplesTable" ref="A4:D15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Client question"/>
     <x:tableColumn id="2" name="Recommended function"/>
@@ -402,7 +402,7 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="VisualIntakeGuideTable" displayName="VisualIntakeGuideTable" ref="A4:C23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="VisualIntakeGuideTable" displayName="VisualIntakeGuideTable" ref="A4:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Capability / decision"/>
     <x:tableColumn id="2" name="Implemented behavior and limits"/>
@@ -808,7 +808,7 @@
         <x:v>Optional image proposals</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
-        <x:v>Visual Intake; seven MCP/API operations, original-image retention, source-only handoff, limits, and unimplemented writes</x:v>
+        <x:v>Visual Intake; nine MCP/API operations, original-image retention, portal/review, and source-only handoff</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -834,7 +834,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1f53e31f1ed40d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3554c99c2478405b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1038,7 +1038,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fcde162345f40d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc4e6ee6fad426f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1182,17 +1182,59 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="33" t="str">
+      <x:c r="A12" s="29" t="str">
         <x:v>Download an Excel account directory or sales report</x:v>
       </x:c>
-      <x:c r="B12" s="34" t="str">
+      <x:c r="B12" s="30" t="str">
         <x:v>create_crm_export</x:v>
       </x:c>
-      <x:c r="C12" s="34" t="str">
+      <x:c r="C12" s="30" t="str">
         <x:v>{"report":"account_directory","format":"xlsx"}</x:v>
       </x:c>
-      <x:c r="D12" s="17" t="str">
+      <x:c r="D12" s="16" t="str">
         <x:v>Creates a bounded immutable workbook with snapshot lineage, row and file checksums, formula-safe cells, expiry, and a short-lived signed URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29" t="str">
+        <x:v>Show quarterly sales by region and customer above a threshold</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>query_business_analytics</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>{"plan":{"dataset":"invoice_sales","dimensions":["invoice_date","region","customer"],"date_grains":{"invoice_date":"quarter"},"metrics":["sales"],"having":{"sales":{"operator":"gte","value":"10000"}},"sort":["invoice_date","-sales"]}}</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="str">
+        <x:v>Typed client-approved semantic model, explicit coverage, currency partition, and no arbitrary SQL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29" t="str">
+        <x:v>Propose an approved contact correction</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="str">
+        <x:v>propose_business_record_change</x:v>
+      </x:c>
+      <x:c r="C14" s="30" t="str">
+        <x:v>Discover the configured object schema, bind the exact prior record SHA-256, and submit a source-cited or user-asserted proposal</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="str">
+        <x:v>The assistant can propose and preview, while operator authorization/apply/reconcile remain separate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="33" t="str">
+        <x:v>Authorize and apply a reviewed record change</x:v>
+      </x:c>
+      <x:c r="B15" s="34" t="str">
+        <x:v>operator JSON API or business_record_changes.py</x:v>
+      </x:c>
+      <x:c r="C15" s="34" t="str">
+        <x:v>An authorized person uses records:authorize, then records:apply and reconciliation against the exact retained authorization</x:v>
+      </x:c>
+      <x:c r="D15" s="17" t="str">
+        <x:v>These routes are intentionally not MCP tools; the assistant cannot self-approve or execute a target write</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1202,7 +1244,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1072c8f788c44295"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43b1bbade6d74e73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1268,7 +1310,7 @@
         <x:v>Local / remote tools</x:v>
       </x:c>
       <x:c r="B7" s="30" t="str">
-        <x:v>12 / 14 default; 19 / up to 21 with intake; remote discovery is scope-filtered</x:v>
+        <x:v>12 / 14 default; 21 / up to 23 with intake; unified client platform supports 29 local / up to 32 remote</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
         <x:v>scripts/ingestion_tools.py</x:v>
@@ -1353,101 +1395,123 @@
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
       <x:c r="A15" s="29" t="str">
-        <x:v>Application API</x:v>
+        <x:v>List sessions</x:v>
       </x:c>
       <x:c r="B15" s="30" t="str">
-        <x:v>POST /api/ingestion/{operation} on remote OAuth server; plain argument JSON. TLS/bearer GET API unchanged</x:v>
+        <x:v>list_ingestion_sessions: owner-scoped paginated recovery</x:v>
       </x:c>
       <x:c r="C15" s="16" t="str">
-        <x:v>references/visual-ingestion.md</x:v>
+        <x:v>ingestion:read</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
       <x:c r="A16" s="29" t="str">
-        <x:v>Limits</x:v>
+        <x:v>Review session</x:v>
       </x:c>
       <x:c r="B16" s="30" t="str">
-        <x:v>1-20 pages/session; PNG/JPEG only; 10,000,000 original bytes and 25,000,000 pixels/page; 1,000,000 JSON bytes/proposal</x:v>
+        <x:v>get_ingestion_review: status and complete proposal receipt history</x:v>
       </x:c>
       <x:c r="C16" s="16" t="str">
-        <x:v>get_ingestion_schema</x:v>
+        <x:v>ingestion:read</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
       <x:c r="A17" s="29" t="str">
-        <x:v>Envelope limit</x:v>
+        <x:v>Application API</x:v>
       </x:c>
       <x:c r="B17" s="30" t="str">
-        <x:v>Remote default 1,000,000 request bytes; --max-request-bytes at least 14,000,000 for maximum image; align proxy/client limits</x:v>
+        <x:v>POST /api/ingestion/{operation} on remote OAuth server; plain argument JSON. TLS/bearer GET API unchanged</x:v>
       </x:c>
       <x:c r="C17" s="16" t="str">
-        <x:v>scripts/retrieval_remote_mcp.py --help</x:v>
+        <x:v>references/visual-ingestion.md</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
       <x:c r="A18" s="29" t="str">
-        <x:v>Correction / retry</x:v>
+        <x:v>Limits</x:v>
       </x:c>
       <x:c r="B18" s="30" t="str">
-        <x:v>Same key and input replays receipt; changed proposal appends under new key. Replacing retained source requires new session</x:v>
+        <x:v>1-20 pages/session; PNG/JPEG only; 10,000,000 original bytes and 25,000,000 pixels/page; 1,000,000 JSON bytes/proposal</x:v>
       </x:c>
       <x:c r="C18" s="16" t="str">
-        <x:v>skills/record-intake/SKILL.md</x:v>
+        <x:v>get_ingestion_schema</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
       <x:c r="A19" s="29" t="str">
-        <x:v>Source-only export</x:v>
+        <x:v>Envelope limit</x:v>
       </x:c>
       <x:c r="B19" s="30" t="str">
-        <x:v>Local visual_ingestion_export.py export / verify retains all originals, proposals and rejections; pins separately retained receipt</x:v>
+        <x:v>Remote default 1,000,000 request bytes; --max-request-bytes at least 14,000,000 for maximum image; align proxy/client limits</x:v>
       </x:c>
       <x:c r="C19" s="16" t="str">
-        <x:v>references/visual-ingestion.md</x:v>
+        <x:v>scripts/retrieval_remote_mcp.py --help</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
       <x:c r="A20" s="29" t="str">
-        <x:v>Prepared source</x:v>
+        <x:v>Correction / retry</x:v>
       </x:c>
       <x:c r="B20" s="30" t="str">
-        <x:v>Complete usable pages get session-named image PDF and page map for normal profiling/intake; blocked or partial PDF cannot advance</x:v>
+        <x:v>Same key and input replays receipt; changed proposal appends under new key. Replacing retained source requires new session</x:v>
       </x:c>
       <x:c r="C20" s="16" t="str">
-        <x:v>visual_intake_source_package_v1</x:v>
+        <x:v>skills/record-intake/SKILL.md</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
       <x:c r="A21" s="29" t="str">
-        <x:v>Publication</x:v>
+        <x:v>Source-only export</x:v>
       </x:c>
       <x:c r="B21" s="30" t="str">
-        <x:v>No proposal promotion, independent-vote conversion, approval, canonical update or live CRM write; business gates still apply</x:v>
+        <x:v>Local visual_ingestion_export.py export / verify retains all originals, proposals and rejections; pins separately retained receipt</x:v>
       </x:c>
       <x:c r="C21" s="16" t="str">
-        <x:v>references/artifact-contracts.md</x:v>
+        <x:v>references/visual-ingestion.md</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
       <x:c r="A22" s="29" t="str">
+        <x:v>Prepared source</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="str">
+        <x:v>Complete usable pages get session-named image PDF and page map for normal profiling/intake; blocked or partial PDF cannot advance</x:v>
+      </x:c>
+      <x:c r="C22" s="16" t="str">
+        <x:v>visual_intake_source_package_v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="54" customHeight="1">
+      <x:c r="A23" s="29" t="str">
+        <x:v>Publication</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>No proposal promotion, independent-vote conversion, approval, canonical update or live CRM write; business gates still apply</x:v>
+      </x:c>
+      <x:c r="C23" s="16" t="str">
+        <x:v>references/artifact-contracts.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="54" customHeight="1">
+      <x:c r="A24" s="29" t="str">
         <x:v>Client support</x:v>
       </x:c>
-      <x:c r="B22" s="30" t="str">
-        <x:v>Actual byte transfer and vision need exact-client acceptance. No bundled capture app, attachment relay or shared review UI</x:v>
-      </x:c>
-      <x:c r="C22" s="16" t="str">
+      <x:c r="B24" s="30" t="str">
+        <x:v>Actual byte transfer and vision need exact-client acceptance. Same-origin portal is bundled; no native chat attachment relay or delegated review role is implied</x:v>
+      </x:c>
+      <x:c r="C24" s="16" t="str">
         <x:v>references/visual-ingestion.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="54" customHeight="1">
-      <x:c r="A23" s="33" t="str">
-        <x:v>Future work</x:v>
-      </x:c>
-      <x:c r="B23" s="34" t="str">
-        <x:v>Governed record create/update, safe general joins, custom metrics and saved reports remain roadmap work</x:v>
-      </x:c>
-      <x:c r="C23" s="17" t="str">
-        <x:v>references/business-data-platform-roadmap.md</x:v>
+    <x:row r="25" ht="54" customHeight="1">
+      <x:c r="A25" s="33" t="str">
+        <x:v>Governed platform</x:v>
+      </x:c>
+      <x:c r="B25" s="34" t="str">
+        <x:v>Client YAML configures typed analytics, saved reports, analytical exports, proposal-only create/amend, plus separately scoped operator API/CLI authorization, apply, and reconciliation; these are not MCP tools</x:v>
+      </x:c>
+      <x:c r="C25" s="17" t="str">
+        <x:v>references/business-data-platform.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1457,7 +1521,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ba708243b9d4cb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc871f1f0115948cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2529,7 +2593,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5b8cea63c114db1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refdeefccd37a4fe3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3104,7 +3168,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f2b1c2cab7e4415"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5dbbd14ef7b427a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3524,7 +3588,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R950fd2af417c4ec1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59627905f61e48b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3623,10 +3687,10 @@
         <x:v>CRM writes</x:v>
       </x:c>
       <x:c r="B8" s="30" t="str">
-        <x:v>No-send common-object import files, target mapping, sandbox proof, authorization, reconciliation, and rollback</x:v>
+        <x:v>No-send common-object files plus governed client-YAML create/amend proposal, authorization, adapter, and reconciliation</x:v>
       </x:c>
       <x:c r="C8" s="30" t="str">
-        <x:v>references/crm-write-readiness.md</x:v>
+        <x:v>references/business-data-platform.md</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
         <x:v>CRM Writes</x:v>
@@ -3637,10 +3701,10 @@
         <x:v>CRM API/MCP</x:v>
       </x:c>
       <x:c r="B9" s="30" t="str">
-        <x:v>Read-only approved-fact discovery, schema, table export, and report functions</x:v>
+        <x:v>Approved-fact retrieval plus optional typed analytics, analytical exports, intake, and record proposals</x:v>
       </x:c>
       <x:c r="C9" s="30" t="str">
-        <x:v>references/canonical-deployment-retrieval.md</x:v>
+        <x:v>references/business-data-platform.md</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
         <x:v>API and MCP</x:v>
@@ -3722,7 +3786,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c869a5c9461410e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca4c651b3bc64b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,9 +4349,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34613817094a46cf"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a26ca3e19644656"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac986d9a9d542b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R633c3ef2ba5f40c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa06891003cf48ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R561350ac77ea4b41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4645,10 +4709,10 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71a5ed65835c4caa"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c649436f997426c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbf2c2aefa964095"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd104362ac2d43cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0135235d876c4141"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ed72bc3a694d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6db95d2a29af4c69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R027f6b6f59834bc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4675,7 +4739,7 @@
     </x:row>
     <x:row r="2" ht="44" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>Approved-data tools share one integrity-checked service. Remote MCP adds owner-bound expiring CSV/XLSX jobs. TLS/bearer REST stays GET-only. Optional source/proposal writes are separate: see Visual Intake.</x:v>
+        <x:v>Approved-data tools share one integrity-checked service. Client YAML adds typed analytics, exports, intake, and record proposals; separately scoped operator API authorization/apply/reconcile is intentionally not MCP. TLS/bearer REST stays GET-only.</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -4713,7 +4777,7 @@
         <x:v>Approved document facts with source citations</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4730,7 +4794,7 @@
         <x:v>One immutable approved document with citation</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4747,7 +4811,7 @@
         <x:v>Routes, tools, reports, and read-only policy</x:v>
       </x:c>
       <x:c r="E7" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4764,7 +4828,7 @@
         <x:v>Batch, registry, source/load hashes, verified table manifests, counts, and reconciliation flags</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4781,7 +4845,7 @@
         <x:v>Declared/extension columns, keys, and available counts</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4798,7 +4862,7 @@
         <x:v>Fast full-text matches across any approved canonical table</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -4815,7 +4879,7 @@
         <x:v>Any canonical row by its single or composite idempotency key</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4832,7 +4896,7 @@
         <x:v>Bounded filters, projection, sorting, and pagination</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4849,7 +4913,7 @@
         <x:v>Checksummed, filtered, paginated approved rows</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4866,7 +4930,7 @@
         <x:v>Party, roles, names, addresses, contacts, activity, currency-separated totals, and source documents</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4883,7 +4947,7 @@
         <x:v>Currency-partitioned sales by company, vendor, region, location, period, ACK, or job</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4900,7 +4964,7 @@
         <x:v>Deterministic source-linked report rows and checksum</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4917,24 +4981,211 @@
         <x:v>Bounded table or standard-report artifact with snapshot lineage, row/file checksums, expiry, and a short-lived signed URL</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
-        <x:v>Additive, non-idempotent report artifact; canonical facts unchanged; no CRM upload</x:v>
+        <x:v>Additive artifact/proposal; canonical facts unchanged; no model authorization</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="33" t="str">
+      <x:c r="A18" s="29" t="str">
         <x:v>Export-job status</x:v>
       </x:c>
-      <x:c r="B18" s="34" t="str">
+      <x:c r="B18" s="30" t="str">
         <x:v>Remote MCP only</x:v>
       </x:c>
-      <x:c r="C18" s="34" t="str">
+      <x:c r="C18" s="30" t="str">
         <x:v>get_crm_export_job</x:v>
       </x:c>
-      <x:c r="D18" s="34" t="str">
+      <x:c r="D18" s="30" t="str">
         <x:v>Owner-bound completed-job metadata, row count, expiry, and checksums</x:v>
       </x:c>
-      <x:c r="E18" s="17" t="str">
-        <x:v>Read-only; approved canonical facts only; no CRM upload</x:v>
+      <x:c r="E18" s="16" t="str">
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="29" t="str">
+        <x:v>Business platform discovery</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>POST /api/platform/get_business_platform_capabilities</x:v>
+      </x:c>
+      <x:c r="C19" s="30" t="str">
+        <x:v>get_business_platform_capabilities</x:v>
+      </x:c>
+      <x:c r="D19" s="30" t="str">
+        <x:v>Configuration fingerprint, enabled datasets/objects/reports, and immutable-snapshot boundary</x:v>
+      </x:c>
+      <x:c r="E19" s="16" t="str">
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="29" t="str">
+        <x:v>Typed analytical query</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="str">
+        <x:v>POST /api/platform/query_business_analytics</x:v>
+      </x:c>
+      <x:c r="C20" s="30" t="str">
+        <x:v>query_business_analytics</x:v>
+      </x:c>
+      <x:c r="D20" s="30" t="str">
+        <x:v>Allowlisted joins, dimensions, metrics, date/fiscal grains, filters, having, totals, sort, pagination, coverage, and checksum</x:v>
+      </x:c>
+      <x:c r="E20" s="16" t="str">
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="29" t="str">
+        <x:v>Saved analytical report</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>POST /api/platform/run_saved_business_report</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>run_saved_business_report</x:v>
+      </x:c>
+      <x:c r="D21" s="30" t="str">
+        <x:v>Client-YAML report plan over the exact approved snapshot</x:v>
+      </x:c>
+      <x:c r="E21" s="16" t="str">
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="29" t="str">
+        <x:v>Analytical CSV/XLSX</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="str">
+        <x:v>POST /api/platform/create_business_analytics_export</x:v>
+      </x:c>
+      <x:c r="C22" s="30" t="str">
+        <x:v>create_business_analytics_export</x:v>
+      </x:c>
+      <x:c r="D22" s="30" t="str">
+        <x:v>Owner-bound expiring checksummed export of one typed plan or saved report</x:v>
+      </x:c>
+      <x:c r="E22" s="16" t="str">
+        <x:v>Additive artifact/proposal; canonical facts unchanged; no model authorization</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="29" t="str">
+        <x:v>Writable object schema</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>POST /api/platform/get_business_object_schema</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>get_business_object_schema</x:v>
+      </x:c>
+      <x:c r="D23" s="30" t="str">
+        <x:v>Configured create/amend fields and explicit no-model-authorization boundary</x:v>
+      </x:c>
+      <x:c r="E23" s="16" t="str">
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="29" t="str">
+        <x:v>Record change proposal</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="str">
+        <x:v>POST /api/platform/propose_business_record_change</x:v>
+      </x:c>
+      <x:c r="C24" s="30" t="str">
+        <x:v>propose_business_record_change</x:v>
+      </x:c>
+      <x:c r="D24" s="30" t="str">
+        <x:v>Append-only owner-scoped proposal receipt; no target or canonical mutation</x:v>
+      </x:c>
+      <x:c r="E24" s="16" t="str">
+        <x:v>Additive artifact/proposal; canonical facts unchanged; no model authorization</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="29" t="str">
+        <x:v>Record change preview</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="str">
+        <x:v>POST /api/platform/preview_business_record_change</x:v>
+      </x:c>
+      <x:c r="C25" s="30" t="str">
+        <x:v>preview_business_record_change</x:v>
+      </x:c>
+      <x:c r="D25" s="30" t="str">
+        <x:v>Snapshot-bound before/after and mapped target payload</x:v>
+      </x:c>
+      <x:c r="E25" s="16" t="str">
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="29" t="str">
+        <x:v>Record change status</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="str">
+        <x:v>POST /api/platform/get_business_record_change</x:v>
+      </x:c>
+      <x:c r="C26" s="30" t="str">
+        <x:v>get_business_record_change</x:v>
+      </x:c>
+      <x:c r="D26" s="30" t="str">
+        <x:v>Integrity-verified proposal and lifecycle receipts without credentials</x:v>
+      </x:c>
+      <x:c r="E26" s="16" t="str">
+        <x:v>Read-only; approved facts or owner-scoped receipts; no CRM upload</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="29" t="str">
+        <x:v>Operator record authorization</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="str">
+        <x:v>POST /api/platform/authorize_business_record_change</x:v>
+      </x:c>
+      <x:c r="C27" s="30" t="str">
+        <x:v>Not exposed to MCP</x:v>
+      </x:c>
+      <x:c r="D27" s="30" t="str">
+        <x:v>records:authorize only; explicit human decision creates an expiring signed authorization</x:v>
+      </x:c>
+      <x:c r="E27" s="16" t="str">
+        <x:v>Separately scoped human/operator API; never callable by the model; canonical facts unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="29" t="str">
+        <x:v>Operator record application</x:v>
+      </x:c>
+      <x:c r="B28" s="30" t="str">
+        <x:v>POST /api/platform/apply_business_record_change</x:v>
+      </x:c>
+      <x:c r="C28" s="30" t="str">
+        <x:v>Not exposed to MCP</x:v>
+      </x:c>
+      <x:c r="D28" s="30" t="str">
+        <x:v>records:apply only; applies one retained authorization through the configured no-send or HTTPS adapter</x:v>
+      </x:c>
+      <x:c r="E28" s="16" t="str">
+        <x:v>Separately scoped human/operator API; never callable by the model; canonical facts unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="33" t="str">
+        <x:v>Operator record reconciliation</x:v>
+      </x:c>
+      <x:c r="B29" s="34" t="str">
+        <x:v>POST /api/platform/reconcile_business_record_change</x:v>
+      </x:c>
+      <x:c r="C29" s="34" t="str">
+        <x:v>Not exposed to MCP</x:v>
+      </x:c>
+      <x:c r="D29" s="34" t="str">
+        <x:v>records:apply only; independently compares every target field and retains mismatches</x:v>
+      </x:c>
+      <x:c r="E29" s="17" t="str">
+        <x:v>Separately scoped human/operator API; never callable by the model; canonical facts unchanged</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4944,7 +5195,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb547f6dbcba24800"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4bf9e5ae15d4fad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5087,7 +5338,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43ff1f76b2b4494d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab46801be3874d47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>